<commit_message>
chore: supplementary documents and figures added, some folder organization updates
</commit_message>
<xml_diff>
--- a/results/04_correlation/Moran_i/moran i_values.xlsx
+++ b/results/04_correlation/Moran_i/moran i_values.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://deepromtech-my.sharepoint.com/personal/bilge_atolyedijital_com_tr/Documents/Desktop/submissions/CIS/repo/04_Correlation/Moran_i/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="180" documentId="11_F25DC773A252ABDACC10489B39DC66C65ADE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DC179E9E-A93F-424E-B8B6-67EAE9FC76EF}"/>
+  <xr:revisionPtr revIDLastSave="212" documentId="11_F25DC773A252ABDACC10489B39DC66C65ADE58E6" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CBDD97C0-388A-4D05-B951-E3D5E506B4DC}"/>
   <bookViews>
-    <workbookView xWindow="2895" yWindow="2895" windowWidth="21600" windowHeight="11190" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Pop_Chg" sheetId="1" r:id="rId1"/>
-    <sheet name="Selected_" sheetId="3" r:id="rId2"/>
+    <sheet name="All Values" sheetId="3" r:id="rId1"/>
+    <sheet name="Pop_Chg" sheetId="1" r:id="rId2"/>
     <sheet name="wd" sheetId="2" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="80">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="82">
   <si>
     <t>Luneburg_Region</t>
   </si>
@@ -248,32 +248,38 @@
     <t>wd</t>
   </si>
   <si>
-    <t>pop 2018</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fac tot </t>
-  </si>
-  <si>
     <t>Pop_chg</t>
   </si>
   <si>
     <t>random</t>
   </si>
   <si>
-    <t>elder</t>
-  </si>
-  <si>
     <t>Lüneburg</t>
   </si>
   <si>
     <t>Lüchow-Dannenberg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Moran_I Values </t>
+  </si>
+  <si>
+    <t>Elder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fac_Tot </t>
+  </si>
+  <si>
+    <t>Pop_2018</t>
+  </si>
+  <si>
+    <t>Supplementary  Table 9: Moran I Results</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -302,6 +308,35 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="9"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -311,7 +346,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -319,11 +354,128 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -340,6 +492,29 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -623,6 +798,180 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{021D8C0D-6C55-4A0E-9A53-968FF7519282}">
+  <dimension ref="A1:K10"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="22.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.140625" customWidth="1"/>
+    <col min="10" max="10" width="39.85546875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:11" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" s="20" t="s">
+        <v>77</v>
+      </c>
+      <c r="B2" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="C2" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="D2" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E2" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="F2" s="22" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" s="23" t="s">
+        <v>42</v>
+      </c>
+      <c r="B3" s="8" t="s">
+        <v>43</v>
+      </c>
+      <c r="C3" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" s="9" t="s">
+        <v>74</v>
+      </c>
+      <c r="F3" s="10" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" s="24" t="s">
+        <v>16</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F4" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A5" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>12</v>
+      </c>
+      <c r="D5" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F5" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A6" s="25" t="s">
+        <v>76</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="14" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F6" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A7" s="24" t="s">
+        <v>22</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="D7" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="E7" s="11" t="s">
+        <v>74</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A8" s="26" t="s">
+        <v>33</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="16" t="s">
+        <v>74</v>
+      </c>
+      <c r="F8" s="17" t="s">
+        <v>74</v>
+      </c>
+      <c r="J8" s="2"/>
+      <c r="K8" s="5"/>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K9" s="4"/>
+    </row>
+    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K10" s="6"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -832,123 +1181,6 @@
       <c r="B14" s="6" t="s">
         <v>43</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{021D8C0D-6C55-4A0E-9A53-968FF7519282}">
-  <dimension ref="A1:K9"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="1" width="39.85546875" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="39.85546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="B1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D1" t="s">
-        <v>74</v>
-      </c>
-      <c r="E1" t="s">
-        <v>75</v>
-      </c>
-      <c r="F1" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>42</v>
-      </c>
-      <c r="B2" s="6" t="s">
-        <v>43</v>
-      </c>
-      <c r="C2" t="s">
-        <v>76</v>
-      </c>
-      <c r="D2" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D4" t="s">
-        <v>76</v>
-      </c>
-      <c r="E4" s="5" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="C5" t="s">
-        <v>76</v>
-      </c>
-      <c r="D5" t="s">
-        <v>76</v>
-      </c>
-      <c r="F5" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="C6" t="s">
-        <v>76</v>
-      </c>
-      <c r="D6" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>33</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" t="s">
-        <v>76</v>
-      </c>
-      <c r="D7" t="s">
-        <v>76</v>
-      </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="5"/>
-    </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="K8" s="4"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
-      <c r="K9" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>